<commit_message>
KFSPTS-37938 Fix template and Remit To Supplier processing
</commit_message>
<xml_diff>
--- a/src/main/resources/edu/cornell/kfs/cemi/vnd/batch/Remit_To_Supplier.xlsx
+++ b/src/main/resources/edu/cornell/kfs/cemi/vnd/batch/Remit_To_Supplier.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30023"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30117"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://huroncg-my.sharepoint.com/personal/thanrahan_huronconsultinggroup_com/Documents/Documents/CloverDX/New Templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cornellprod.sharepoint.com/sites/CEMI-DOC/CEMI_Library_Draft/Projects/ERP/05 - Technical Vertical/Data_Conversion/A&amp;C/Workset A Templates with Mapping Notes/SCM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{65C67EF3-7CF7-47F4-91D0-C0CD88B7F085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F6419A6D-85A0-494C-9834-81B7D1D8A8AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Remit_To_Supplier" sheetId="6" r:id="rId1"/>
-    <sheet name="Remit_To_Supplier_FULL" sheetId="1" r:id="rId2"/>
+    <sheet name="Remit_To_Supplier_FULL" sheetId="1" state="hidden" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -70,7 +70,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C5" authorId="0" shapeId="0" xr:uid="{B003BCF0-6E78-4A9E-BF2B-D9D31D609854}">
+    <comment ref="C5" authorId="0" shapeId="0" xr:uid="{AA24A7CC-B823-4905-85DF-B875E85A702C}">
       <text>
         <r>
           <rPr>
@@ -84,7 +84,21 @@
         </r>
       </text>
     </comment>
-    <comment ref="D5" authorId="0" shapeId="0" xr:uid="{C5DC0139-2AA9-497B-A37F-29E28A3D4294}">
+    <comment ref="D5" authorId="0" shapeId="0" xr:uid="{B003BCF0-6E78-4A9E-BF2B-D9D31D609854}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color indexed="8"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Text item</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E5" authorId="0" shapeId="0" xr:uid="{C5DC0139-2AA9-497B-A37F-29E28A3D4294}">
       <text>
         <r>
           <rPr>
@@ -98,7 +112,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E5" authorId="0" shapeId="0" xr:uid="{E47966ED-1D4F-46B1-BE2C-BA09DFBE254F}">
+    <comment ref="F5" authorId="0" shapeId="0" xr:uid="{E47966ED-1D4F-46B1-BE2C-BA09DFBE254F}">
       <text>
         <r>
           <rPr>
@@ -112,7 +126,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F5" authorId="0" shapeId="0" xr:uid="{FAD3F247-3000-476A-BA55-9B69869CEFB0}">
+    <comment ref="G5" authorId="0" shapeId="0" xr:uid="{FAD3F247-3000-476A-BA55-9B69869CEFB0}">
       <text>
         <r>
           <rPr>
@@ -126,7 +140,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G5" authorId="0" shapeId="0" xr:uid="{96D2B346-F264-417A-9170-D2653BE4D185}">
+    <comment ref="H5" authorId="0" shapeId="0" xr:uid="{96D2B346-F264-417A-9170-D2653BE4D185}">
       <text>
         <r>
           <rPr>
@@ -140,7 +154,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H5" authorId="0" shapeId="0" xr:uid="{8C7BD76F-F24D-4694-B3AC-F01E32236B23}">
+    <comment ref="I5" authorId="0" shapeId="0" xr:uid="{8C7BD76F-F24D-4694-B3AC-F01E32236B23}">
       <text>
         <r>
           <rPr>
@@ -154,7 +168,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I5" authorId="0" shapeId="0" xr:uid="{B3B13686-6BC6-4112-8C38-3A8C94FD8BCE}">
+    <comment ref="J5" authorId="0" shapeId="0" xr:uid="{B3B13686-6BC6-4112-8C38-3A8C94FD8BCE}">
       <text>
         <r>
           <rPr>
@@ -168,7 +182,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J5" authorId="0" shapeId="0" xr:uid="{0191CD26-F2C8-424A-A510-79EBCEAA5551}">
+    <comment ref="K5" authorId="0" shapeId="0" xr:uid="{0191CD26-F2C8-424A-A510-79EBCEAA5551}">
       <text>
         <r>
           <rPr>
@@ -182,7 +196,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K5" authorId="0" shapeId="0" xr:uid="{08BA44E8-AF85-451E-9F7B-7270CA650C16}">
+    <comment ref="L5" authorId="0" shapeId="0" xr:uid="{08BA44E8-AF85-451E-9F7B-7270CA650C16}">
       <text>
         <r>
           <rPr>
@@ -196,7 +210,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L5" authorId="0" shapeId="0" xr:uid="{EAF5D1AB-C3B1-4727-B3AD-E6E1F950E95B}">
+    <comment ref="M5" authorId="0" shapeId="0" xr:uid="{EAF5D1AB-C3B1-4727-B3AD-E6E1F950E95B}">
       <text>
         <r>
           <rPr>
@@ -210,7 +224,21 @@
         </r>
       </text>
     </comment>
-    <comment ref="M5" authorId="0" shapeId="0" xr:uid="{45F97B1D-8046-420D-B43E-AFE663782CCB}">
+    <comment ref="N5" authorId="0" shapeId="0" xr:uid="{0EF7571A-3543-4D93-AC6B-45C7482C5C54}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color indexed="8"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Text item</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O5" authorId="0" shapeId="0" xr:uid="{45F97B1D-8046-420D-B43E-AFE663782CCB}">
       <text>
         <r>
           <rPr>
@@ -224,7 +252,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N5" authorId="0" shapeId="0" xr:uid="{C1633A83-EDB5-4DC8-A105-9062E1AEA749}">
+    <comment ref="P5" authorId="0" shapeId="0" xr:uid="{C1633A83-EDB5-4DC8-A105-9062E1AEA749}">
       <text>
         <r>
           <rPr>
@@ -238,7 +266,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O5" authorId="0" shapeId="0" xr:uid="{68B1F809-75F5-4790-872F-B692FE102434}">
+    <comment ref="Q5" authorId="0" shapeId="0" xr:uid="{68B1F809-75F5-4790-872F-B692FE102434}">
       <text>
         <r>
           <rPr>
@@ -266,7 +294,21 @@
         </r>
       </text>
     </comment>
-    <comment ref="C6" authorId="0" shapeId="0" xr:uid="{10119193-51C6-4A56-B143-E71160FAC288}">
+    <comment ref="C6" authorId="0" shapeId="0" xr:uid="{F2AF8EA2-16D2-4A71-B70D-8EAE00763C51}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color indexed="8"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Supplier Connection ID</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D6" authorId="0" shapeId="0" xr:uid="{10119193-51C6-4A56-B143-E71160FAC288}">
       <text>
         <r>
           <rPr>
@@ -280,7 +322,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D6" authorId="0" shapeId="0" xr:uid="{4805AC85-7DE8-48BE-9282-4EEB8363A190}">
+    <comment ref="E6" authorId="0" shapeId="0" xr:uid="{4805AC85-7DE8-48BE-9282-4EEB8363A190}">
       <text>
         <r>
           <rPr>
@@ -294,7 +336,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E6" authorId="0" shapeId="0" xr:uid="{EA137665-E544-462F-AC9E-EC82F3641D4D}">
+    <comment ref="F6" authorId="0" shapeId="0" xr:uid="{EA137665-E544-462F-AC9E-EC82F3641D4D}">
       <text>
         <r>
           <rPr>
@@ -308,7 +350,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F6" authorId="0" shapeId="0" xr:uid="{FCAAFBEB-44A6-4735-85C6-E0A591980EE2}">
+    <comment ref="G6" authorId="0" shapeId="0" xr:uid="{FCAAFBEB-44A6-4735-85C6-E0A591980EE2}">
       <text>
         <r>
           <rPr>
@@ -322,7 +364,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G6" authorId="0" shapeId="0" xr:uid="{380C0531-9F44-4065-938A-FF44294F1DA9}">
+    <comment ref="H6" authorId="0" shapeId="0" xr:uid="{380C0531-9F44-4065-938A-FF44294F1DA9}">
       <text>
         <r>
           <rPr>
@@ -336,7 +378,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H6" authorId="0" shapeId="0" xr:uid="{F97B165C-1932-4AA4-96BC-3432B6C7EBC7}">
+    <comment ref="I6" authorId="0" shapeId="0" xr:uid="{F97B165C-1932-4AA4-96BC-3432B6C7EBC7}">
       <text>
         <r>
           <rPr>
@@ -350,7 +392,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I6" authorId="0" shapeId="0" xr:uid="{57032E46-B0FE-4EEC-A530-E784B2332D7D}">
+    <comment ref="J6" authorId="0" shapeId="0" xr:uid="{57032E46-B0FE-4EEC-A530-E784B2332D7D}">
       <text>
         <r>
           <rPr>
@@ -364,7 +406,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J6" authorId="0" shapeId="0" xr:uid="{A6250C54-52E9-4843-8CAF-78321B683EEF}">
+    <comment ref="K6" authorId="0" shapeId="0" xr:uid="{A6250C54-52E9-4843-8CAF-78321B683EEF}">
       <text>
         <r>
           <rPr>
@@ -378,7 +420,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K6" authorId="0" shapeId="0" xr:uid="{CE0C6FBC-D948-4477-842A-66C90DFD5A4D}">
+    <comment ref="L6" authorId="0" shapeId="0" xr:uid="{CE0C6FBC-D948-4477-842A-66C90DFD5A4D}">
       <text>
         <r>
           <rPr>
@@ -392,7 +434,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L6" authorId="0" shapeId="0" xr:uid="{092F0F8B-EAE0-49A7-B976-275021313DC6}">
+    <comment ref="M6" authorId="0" shapeId="0" xr:uid="{092F0F8B-EAE0-49A7-B976-275021313DC6}">
       <text>
         <r>
           <rPr>
@@ -406,7 +448,21 @@
         </r>
       </text>
     </comment>
-    <comment ref="M6" authorId="0" shapeId="0" xr:uid="{905D44DC-3442-45AD-BA36-A49771940511}">
+    <comment ref="N6" authorId="0" shapeId="0" xr:uid="{CB712EA5-1560-42BE-8929-5069E23C8E3B}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color indexed="8"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Payment Memo for the Supplier Connection</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O6" authorId="0" shapeId="0" xr:uid="{905D44DC-3442-45AD-BA36-A49771940511}">
       <text>
         <r>
           <rPr>
@@ -420,7 +476,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N6" authorId="0" shapeId="0" xr:uid="{EBAB1DB4-C907-4B8D-A6FC-73850DCF3EF5}">
+    <comment ref="P6" authorId="0" shapeId="0" xr:uid="{EBAB1DB4-C907-4B8D-A6FC-73850DCF3EF5}">
       <text>
         <r>
           <rPr>
@@ -434,7 +490,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O6" authorId="0" shapeId="0" xr:uid="{1955C16B-F4A2-40A4-8D53-7C16C1B6A09B}">
+    <comment ref="Q6" authorId="0" shapeId="0" xr:uid="{1955C16B-F4A2-40A4-8D53-7C16C1B6A09B}">
       <text>
         <r>
           <rPr>
@@ -1311,7 +1367,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="78">
   <si>
     <t>Submit Remit To Supplier Connection</t>
   </si>
@@ -1363,6 +1419,9 @@
     <t>Required</t>
   </si>
   <si>
+    <t>Optional</t>
+  </si>
+  <si>
     <t>Required. May have multiples</t>
   </si>
   <si>
@@ -1372,9 +1431,6 @@
     <t>CondRequired</t>
   </si>
   <si>
-    <t>Optional</t>
-  </si>
-  <si>
     <t>Format</t>
   </si>
   <si>
@@ -1405,6 +1461,9 @@
     <t>Supplier</t>
   </si>
   <si>
+    <t>Supplier_Connection_ID</t>
+  </si>
+  <si>
     <t>Supplier_Connection_Name</t>
   </si>
   <si>
@@ -1435,6 +1494,9 @@
     <t>Alternate_Name_Usage</t>
   </si>
   <si>
+    <t>Payment_Memo</t>
+  </si>
+  <si>
     <t>Is_Default</t>
   </si>
   <si>
@@ -1465,9 +1527,6 @@
     <t>Supplier_Reference_ID</t>
   </si>
   <si>
-    <t>Supplier_Connection_ID</t>
-  </si>
-  <si>
     <t>Remit_To_Supplier</t>
   </si>
   <si>
@@ -1490,9 +1549,6 @@
   </si>
   <si>
     <t>Accepted_Payment_Type_10</t>
-  </si>
-  <si>
-    <t>Payment_Memo</t>
   </si>
   <si>
     <t>Default_Currency</t>
@@ -1649,7 +1705,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -1681,12 +1737,79 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1705,11 +1828,20 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2028,151 +2160,166 @@
   <sheetPr>
     <tabColor theme="0" tint="-0.14999847407452621"/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <dimension ref="A1:Q6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="21.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="24.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="17.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="20.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="32.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="25.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="26.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="31.140625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="33" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="20.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="43.5703125" customWidth="1"/>
+    <col min="2" max="2" width="27.7109375" customWidth="1"/>
+    <col min="3" max="3" width="40.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="32.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="31.140625" customWidth="1"/>
+    <col min="15" max="15" width="33" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="41.85546875" customWidth="1"/>
+    <col min="17" max="17" width="20.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="91.5">
+    <row r="1" spans="1:17" ht="91.5">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="18"/>
+      <c r="D1" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12" t="s">
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="J1" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="K1" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="K1" s="12" t="s">
+      <c r="L1" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="L1" s="12" t="s">
+      <c r="M1" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="M1" s="12" t="s">
+      <c r="N1" s="18"/>
+      <c r="O1" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="N1" s="12" t="s">
+      <c r="P1" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="O1" s="12"/>
+      <c r="Q1" s="18"/>
     </row>
-    <row r="2" spans="1:15" ht="17.45">
-      <c r="A2" s="11" t="s">
+    <row r="2" spans="1:17" ht="108.75" customHeight="1">
+      <c r="A2" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-      <c r="N2" s="12"/>
-      <c r="O2" s="12"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="16"/>
+      <c r="P2" s="16"/>
+      <c r="Q2" s="16"/>
     </row>
-    <row r="3" spans="1:15" ht="17.45">
+    <row r="3" spans="1:17" ht="18">
       <c r="A3" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="10"/>
-      <c r="M3" s="10"/>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
+      <c r="D3" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="21"/>
+      <c r="L3" s="21"/>
+      <c r="M3" s="21"/>
+      <c r="N3" s="21"/>
+      <c r="O3" s="21"/>
+      <c r="P3" s="21"/>
+      <c r="Q3" s="21"/>
     </row>
-    <row r="4" spans="1:15" ht="17.45">
+    <row r="4" spans="1:17" ht="18">
       <c r="A4" s="13" t="s">
         <v>14</v>
       </c>
       <c r="B4" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="9" t="s">
-        <v>15</v>
+      <c r="C4" s="7" t="s">
+        <v>16</v>
       </c>
       <c r="D4" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E4" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="J4" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="K4" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="H4" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="I4" s="9" t="s">
+      <c r="L4" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="M4" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="N4" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="O4" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="J4" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="K4" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="L4" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="M4" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="N4" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="O4" s="7" t="s">
-        <v>19</v>
+      <c r="P4" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q4" s="7" t="s">
+        <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="17.45">
+    <row r="5" spans="1:17" ht="18">
       <c r="A5" s="13" t="s">
         <v>20</v>
       </c>
@@ -2183,7 +2330,7 @@
         <v>22</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>23</v>
@@ -2195,10 +2342,10 @@
         <v>23</v>
       </c>
       <c r="H5" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="I5" s="7" t="s">
         <v>24</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>22</v>
       </c>
       <c r="J5" s="7" t="s">
         <v>22</v>
@@ -2207,19 +2354,25 @@
         <v>22</v>
       </c>
       <c r="L5" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="M5" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="M5" s="7" t="s">
-        <v>26</v>
-      </c>
       <c r="N5" s="7" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="O5" s="7" t="s">
         <v>26</v>
       </c>
+      <c r="P5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q5" s="7" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="6" spans="1:15" ht="17.45">
+    <row r="6" spans="1:17" ht="18">
       <c r="A6" s="13" t="s">
         <v>28</v>
       </c>
@@ -2265,46 +2418,36 @@
       <c r="O6" s="6" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="7" spans="1:15">
-      <c r="A7" s="14"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="14"/>
-      <c r="M7" s="4"/>
-      <c r="N7" s="4"/>
-      <c r="O7" s="4"/>
-    </row>
-    <row r="8" spans="1:15">
-      <c r="O8" s="4"/>
+      <c r="P6" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q6" s="6" t="s">
+        <v>44</v>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="M7:M1048576 O7:O1048576" xr:uid="{3DEC6EB0-3195-4A4B-83FE-2E1F12FD1ADE}">
+  <dataValidations count="8">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="Q17:Q1048576 O17:O1048576" xr:uid="{3DEC6EB0-3195-4A4B-83FE-2E1F12FD1ADE}">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="N5" xr:uid="{9BE51DEE-584F-4223-B858-7364166680F6}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="P5" xr:uid="{9BE51DEE-584F-4223-B858-7364166680F6}">
       <formula1>"WID,Payment_Terms_ID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L5" xr:uid="{B63F7DDD-512C-421A-9E0B-A7C78E914398}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="M5" xr:uid="{B63F7DDD-512C-421A-9E0B-A7C78E914398}">
       <formula1>"Alternate_Name_Usage_ID,WID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H5" xr:uid="{04450BFE-489B-4E95-9535-97B7B4645901}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I5" xr:uid="{04450BFE-489B-4E95-9535-97B7B4645901}">
       <formula1>"WID,Payee_Settlement_Bank_Account_ID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D5:G5" xr:uid="{E95B4EEA-BAB0-4CD6-9AE6-8F16FB7462B7}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E5:H5" xr:uid="{E95B4EEA-BAB0-4CD6-9AE6-8F16FB7462B7}">
       <formula1>"Payment_Type_ID,WID"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B5" xr:uid="{762E3225-3CCF-46F1-B931-5189DD6B8319}">
       <formula1>"WID,Supplier_ID,External_Sourceable_ID,Supplier_Reference_ID"</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A7:C9 E7:E9 F9:H9 L7:XFD9 I7 I8:I9 J9:K9" xr:uid="{FDE4197E-1935-4A0F-91A7-7E37CAA514B7}"/>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="AD10:AE16 AA10:AA16" xr:uid="{604E170F-A8B7-471B-A0BB-B47A69077AD5}">
+      <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2350,16 +2493,16 @@
       <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
       <c r="E1" s="12" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H1" s="12"/>
       <c r="I1" s="12"/>
@@ -2395,15 +2538,15 @@
         <v>9</v>
       </c>
       <c r="AA1" s="12" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="AB1" s="12"/>
       <c r="AC1" s="12"/>
       <c r="AD1" s="12" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:30" ht="17.45">
+    <row r="2" spans="1:30" ht="18">
       <c r="A2" s="11" t="s">
         <v>10</v>
       </c>
@@ -2437,7 +2580,7 @@
       <c r="AC2" s="12"/>
       <c r="AD2" s="12"/>
     </row>
-    <row r="3" spans="1:30" ht="17.45">
+    <row r="3" spans="1:30" ht="18">
       <c r="A3" s="13" t="s">
         <v>11</v>
       </c>
@@ -2475,7 +2618,7 @@
       <c r="AC3" s="10"/>
       <c r="AD3" s="10"/>
     </row>
-    <row r="4" spans="1:30" ht="17.45">
+    <row r="4" spans="1:30" ht="18">
       <c r="A4" s="13" t="s">
         <v>14</v>
       </c>
@@ -2483,13 +2626,13 @@
         <v>15</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>15</v>
@@ -2501,73 +2644,73 @@
         <v>15</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="O4" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="P4" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="Q4" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="R4" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="S4" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="T4" s="9" t="s">
         <v>15</v>
       </c>
       <c r="U4" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="V4" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="V4" s="9" t="s">
-        <v>18</v>
-      </c>
       <c r="W4" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X4" s="7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="Y4" s="9" t="s">
         <v>15</v>
       </c>
       <c r="Z4" s="7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="AA4" s="7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="AB4" s="7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="AC4" s="7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="AD4" s="9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:30" ht="17.45">
+    <row r="5" spans="1:30" ht="18">
       <c r="A5" s="13" t="s">
         <v>20</v>
       </c>
@@ -2647,7 +2790,7 @@
         <v>27</v>
       </c>
       <c r="AA5" s="7" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AB5" s="7" t="s">
         <v>26</v>
@@ -2656,10 +2799,10 @@
         <v>26</v>
       </c>
       <c r="AD5" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:30" ht="17.45">
+    <row r="6" spans="1:30" ht="18">
       <c r="A6" s="13" t="s">
         <v>28</v>
       </c>
@@ -2667,82 +2810,82 @@
         <v>29</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>21</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="N6" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q6" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="R6" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="S6" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="T6" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="U6" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V6" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W6" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="X6" s="6" t="s">
-        <v>59</v>
+        <v>41</v>
       </c>
       <c r="Y6" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="Z6" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="AA6" s="6" t="s">
         <v>60</v>
       </c>
       <c r="AB6" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="AC6" s="6" t="s">
         <v>61</v>
@@ -2824,7 +2967,7 @@
       <c r="X7" s="2" t="s" cm="1">
         <v>64</v>
       </c>
-      <c r="Y7" s="16" t="b">
+      <c r="Y7" s="15" t="b">
         <v>1</v>
       </c>
       <c r="Z7" s="2" t="s" cm="1">
@@ -2836,7 +2979,7 @@
       <c r="AB7" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AC7" s="16" t="b">
+      <c r="AC7" s="15" t="b">
         <v>1</v>
       </c>
       <c r="AD7" s="2" t="s">
@@ -2945,21 +3088,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="d8c1821b-25b7-4bd3-913e-b4d27807b973" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Phase xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
-    <Vertical xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
-    <ProjectPhase xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
-    <Owner xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
-    <Comments xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
-    <ContentDate xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
-    <Status xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04">Draft</Status>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3235,16 +3369,25 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="d8c1821b-25b7-4bd3-913e-b4d27807b973" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Phase xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
+    <Vertical xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
+    <ProjectPhase xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
+    <Owner xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
+    <Comments xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
+    <ContentDate xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
+    <Status xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04">Draft</Status>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2F1CEAD1-1CB6-4053-8EE7-630E68731F85}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{371A7E7F-7040-4721-8A7B-7330029622EF}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3252,5 +3395,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{371A7E7F-7040-4721-8A7B-7330029622EF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2F1CEAD1-1CB6-4053-8EE7-630E68731F85}"/>
 </file>
</xml_diff>